<commit_message>
Save library recording Session 13/10/2026, 08:03:59 - 65172bf1-fd13-4458-a189-401a8bbd20dd - 2026-10-12T21:09:02.217861Z
</commit_message>
<xml_diff>
--- a/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/65172bf1-fd13-4458-a189-401a8bbd20dd/resources/azure-devops.xlsx
+++ b/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/65172bf1-fd13-4458-a189-401a8bbd20dd/resources/azure-devops.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,6 +448,538 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Open https://hfm-wholesale-app-dev.ashysand-8cabb4df.australiaeast.azurecontainerapps.io/daily-orders?storeNo=426&amp;date=2026-10-08</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://hfm-wholesale-app-dev.ashysand-8cabb4df.australiaeast.azurecontainerapps.io/daily-orders?storeNo=426&amp;date=2026-10-08</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Click 152,303</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(1) &gt; input:nth-of-type(1)", "x": 152, "y": 303, "text": "", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>step-002.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Type: Sa</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sa</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(1) &gt; input:nth-of-type(1)"}</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>step-003.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Click DEV
+Wholesale sign in
+Use the account details issued for your store.
+* Require</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>{"primary": "#root &gt; div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1)", "x": 146, "y": 418, "text": "DEV\nWholesale sign in\n\nUse the account details issued for your store.\n\n* Require", "tag": "form"}</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>step-004.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Click 212,408</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(2) &gt; input:nth-of-type(1)", "x": 212, "y": 408, "text": "", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>step-005.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Type: {{HFM_Ext_pass}}</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>{{HFM_Ext_pass}}</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(2) &gt; input:nth-of-type(1)"}</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>step-006.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Click Sign in</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>{"primary": "#root &gt; div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; button:nth-of-type(1)", "x": 204, "y": 519, "text": "Sign in", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>step-007.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Click HFM Internal Production</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>{"primary": "main:nth-of-type(1) &gt; section:nth-of-type(1) &gt; div:nth-of-type(3) &gt; div:nth-of-type(1) &gt; div:nth-of-type(1) &gt; select:nth-of-type(1)", "x": 126, "y": 260, "text": "HFM Internal Production", "tag": "select"}</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>step-008.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Type: Hi-Tech</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Hi-Tech</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>{"primary": "input[placeholder=\"Search stores\"]"}</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>step-009.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Click Hi-Tech
+Store 426</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>{"primary": "#\\:r2\\: &gt; button:nth-of-type(1)", "x": 118, "y": 381, "text": "Hi-Tech\nStore 426", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>step-010.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Click Ordered quantity for ASIAN - BABY / SHANGHI BOK CHOY</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>{"primary": "input[aria-label=\"Ordered quantity for ASIAN - BABY / SHANGHI BOK CHOY\"]", "x": 654, "y": 407, "text": "Ordered quantity for ASIAN - BABY / SHANGHI BOK CHOY", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>step-011.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Click 649,420</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>{"primary": "section:nth-of-type(1) &gt; div:nth-of-type(4) &gt; table:nth-of-type(1) &gt; tbody:nth-of-type(1) &gt; tr:nth-of-type(1) &gt; td:nth-of-type(6)", "x": 649, "y": 420, "text": "", "tag": "td"}</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>step-012.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Click Ordered quantity for ASIAN - BABY / SHANGHI BOK CHOY</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>{"primary": "input[aria-label=\"Ordered quantity for ASIAN - BABY / SHANGHI BOK CHOY\"]", "x": 638, "y": 396, "text": "Ordered quantity for ASIAN - BABY / SHANGHI BOK CHOY", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>step-013.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Type: 2</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(4) &gt; table:nth-of-type(1) &gt; tbody:nth-of-type(1) &gt; tr:nth-of-type(1) &gt; td:nth-of-type(6) &gt; input:nth-of-type(1)"}</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>step-014.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Click Comment for ASIAN - BABY / SHANGHI BOK CHOY</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>{"primary": "input[aria-label=\"Comment for ASIAN - BABY / SHANGHI BOK CHOY\"]", "x": 889, "y": 404, "text": "Comment for ASIAN - BABY / SHANGHI BOK CHOY", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>step-015.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Type: Test order ignore</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Test order ignore</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>step-016.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Click 829,165</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>{"primary": "#\\:r0\\:-1312\\%7C51-comment", "x": 829, "y": 165, "text": "", "tag": "td"}</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>step-017.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Session 13/10/2026, 08:03:59</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Press ArrowUp ×18</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ArrowUp</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>step-018.png</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Save library recording Session 13/10/2026, 08:03:59 - 65172bf1-fd13-4458-a189-401a8bbd20dd - 2026-10-12T21:11:22.507185Z
</commit_message>
<xml_diff>
--- a/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/65172bf1-fd13-4458-a189-401a8bbd20dd/resources/azure-devops.xlsx
+++ b/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/65172bf1-fd13-4458-a189-401a8bbd20dd/resources/azure-devops.xlsx
@@ -466,7 +466,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://hfm-wholesale-app-dev.ashysand-8cabb4df.australiaeast.azurecontainerapps.io/daily-orders?storeNo=426&amp;date=2026-10-08</t>
+          <t>https://hfm-wholesale-app-dev.ashysand-8cabb4df.australiaeast.azurecontainerapps.io/daily-orders?storeNo=4{{Order_Qty}}6&amp;date={{Order_Qty}}0{{Order_Qty}}6-10-08</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -522,7 +522,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sa</t>
+          <t>{{Ext_User_ID}}</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Hi-Tech</t>
+          <t>{{placeholder_stores1}}</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>{{Order_Qty}}</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Test order ignore</t>
+          <t>{{Orser_commwnta}}</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">

</xml_diff>

<commit_message>
Save library recording Session 13/10/2026, 08:03:59 - 65172bf1-fd13-4458-a189-401a8bbd20dd - 2026-10-12T21:14:39.806535Z
</commit_message>
<xml_diff>
--- a/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/65172bf1-fd13-4458-a189-401a8bbd20dd/resources/azure-devops.xlsx
+++ b/library/projects/1c7a86a9-9525-4bd4-b5f0-df360a7b49f1/recordings/65172bf1-fd13-4458-a189-401a8bbd20dd/resources/azure-devops.xlsx
@@ -495,7 +495,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(1) &gt; input:nth-of-type(1)", "x": 152, "y": 303, "text": "", "tag": "input"}</t>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(1) &gt; input:nth-of-type(1)", "tag": "input", "text": "", "x": 152, "y": 303}</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -558,7 +558,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>{"primary": "#root &gt; div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1)", "x": 146, "y": 418, "text": "DEV\nWholesale sign in\n\nUse the account details issued for your store.\n\n* Require", "tag": "form"}</t>
+          <t>{"primary": "#root &gt; div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1)", "tag": "form", "text": "DEV\nWholesale sign in\n\nUse the account details issued for your store.\n\n* Require", "x": 146, "y": 418}</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -586,7 +586,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(2) &gt; input:nth-of-type(1)", "x": 212, "y": 408, "text": "", "tag": "input"}</t>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; label:nth-of-type(2) &gt; input:nth-of-type(1)", "tag": "input", "text": "", "x": 212, "y": 408}</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -646,7 +646,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>{"primary": "#root &gt; div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; button:nth-of-type(1)", "x": 204, "y": 519, "text": "Sign in", "tag": "button"}</t>
+          <t>{"primary": "#root &gt; div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; form:nth-of-type(1) &gt; button:nth-of-type(1)", "tag": "button", "text": "Sign in", "x": 204, "y": 519}</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -674,7 +674,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>{"primary": "main:nth-of-type(1) &gt; section:nth-of-type(1) &gt; div:nth-of-type(3) &gt; div:nth-of-type(1) &gt; div:nth-of-type(1) &gt; select:nth-of-type(1)", "x": 126, "y": 260, "text": "HFM Internal Production", "tag": "select"}</t>
+          <t>{"primary": "main:nth-of-type(1) &gt; section:nth-of-type(1) &gt; div:nth-of-type(3) &gt; div:nth-of-type(1) &gt; div:nth-of-type(1) &gt; select:nth-of-type(1)", "tag": "select", "text": "HFM Internal Production", "x": 126, "y": 260}</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -735,7 +735,7 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>{"primary": "#\\:r2\\: &gt; button:nth-of-type(1)", "x": 118, "y": 381, "text": "Hi-Tech\nStore 426", "tag": "button"}</t>
+          <t>{"primary": "#\\:r2\\: &gt; button:nth-of-type(1)", "tag": "button", "text": "Hi-Tech\nStore 426", "x": 118, "y": 381}</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -763,7 +763,7 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>{"primary": "input[aria-label=\"Ordered quantity for ASIAN - BABY / SHANGHI BOK CHOY\"]", "x": 654, "y": 407, "text": "Ordered quantity for ASIAN - BABY / SHANGHI BOK CHOY", "tag": "input"}</t>
+          <t>{"primary": "input[aria-label=\"Ordered quantity for ASIAN - BABY / SHANGHI BOK CHOY\"]", "tag": "input", "text": "Ordered quantity for ASIAN - BABY / SHANGHI BOK CHOY", "x": 654, "y": 407}</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -791,7 +791,7 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>{"primary": "section:nth-of-type(1) &gt; div:nth-of-type(4) &gt; table:nth-of-type(1) &gt; tbody:nth-of-type(1) &gt; tr:nth-of-type(1) &gt; td:nth-of-type(6)", "x": 649, "y": 420, "text": "", "tag": "td"}</t>
+          <t>{"primary": "section:nth-of-type(1) &gt; div:nth-of-type(4) &gt; table:nth-of-type(1) &gt; tbody:nth-of-type(1) &gt; tr:nth-of-type(1) &gt; td:nth-of-type(6)", "tag": "td", "text": "", "x": 649, "y": 420}</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -819,7 +819,7 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>{"primary": "input[aria-label=\"Ordered quantity for ASIAN - BABY / SHANGHI BOK CHOY\"]", "x": 638, "y": 396, "text": "Ordered quantity for ASIAN - BABY / SHANGHI BOK CHOY", "tag": "input"}</t>
+          <t>{"primary": "input[aria-label=\"Ordered quantity for ASIAN - BABY / SHANGHI BOK CHOY\"]", "tag": "input", "text": "Ordered quantity for ASIAN - BABY / SHANGHI BOK CHOY", "x": 638, "y": 396}</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -879,7 +879,7 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>{"primary": "input[aria-label=\"Comment for ASIAN - BABY / SHANGHI BOK CHOY\"]", "x": 889, "y": 404, "text": "Comment for ASIAN - BABY / SHANGHI BOK CHOY", "tag": "input"}</t>
+          <t>{"primary": "input[aria-label=\"Comment for ASIAN - BABY / SHANGHI BOK CHOY\"]", "tag": "input", "text": "Comment for ASIAN - BABY / SHANGHI BOK CHOY", "x": 889, "y": 404}</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -939,7 +939,7 @@
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>{"primary": "#\\:r0\\:-1312\\%7C51-comment", "x": 829, "y": 165, "text": "", "tag": "td"}</t>
+          <t>{"primary": "#\\:r0\\:-1312\\%7C51-comment", "tag": "td", "text": "", "x": 829, "y": 165}</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">

</xml_diff>